<commit_message>
fix(evidence): clarify observations and preserve bounded model evidence
</commit_message>
<xml_diff>
--- a/docs/labels-review.xlsx
+++ b/docs/labels-review.xlsx
@@ -489,19 +489,19 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Labels are where an investigation starts. The report lays every label of every node out as worth opening, worth noticing, or ordinary; `mongo-log-parser label &lt;bundle&gt; &lt;label&gt; --source &lt;node&gt;` opens one: the exact seconds it was past its mark, the labels it pairs with over those seconds, and the node's log in the same window.</t>
+          <t>Labels summarize observations and guide navigation, not causes or fixes. The report uses fixed review references to group findings. Opening a label shows observed samples and timestamps, paired measurements and available matched-node logs. Legacy label IDs are stable identifiers, not proof of their implied condition.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>One second</t>
+          <t>One sample</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>FTDC samples about once a second. "What one second is" is the formula for each sample. Δ is a counter read as its change a second.</t>
+          <t>FTDC commonly samples about once a second, but cadence and gaps must be checked. Formulas apply to available samples. Counter rates use elapsed time; sample counts are not continuous elapsed durations.</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Each minute keeps its mean, its highest and lowest second, and — for a rule with a threshold — how many seconds were past it. "Read on" is the summary the bands and the shape use. A burst that a minute mean would hide (a ticket pool empty for ten seconds) is counted in seconds (s/min) instead.</t>
+          <t>Minute summaries keep the mean and extreme valid samples. Time views normalize the share of valid samples past a fixed reference to 60 s/min; this is not continuous elapsed time. A binned chart extremum does not show how long it persisted.</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Fuzzy: a value near an edge belongs to two bands by degree. "Example" shows one such value.</t>
+          <t>Fixed descriptive references, not incident severity, discovered limits or diagnostic confidence. Fuzzy membership means a value can belong to two bands by degree. "Example" shows one such value.</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The band from which the label is listed as worth opening. The default is the top two bands of four or more, the top band otherwise; a rule can lower it (a single second with no ticket left is worth opening).</t>
+          <t>Fixed navigation rule: the top two of four or more bands, or the top band otherwise. Definitions may choose another review band, including one isolated sample. This ranking does not establish impact or cause.</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Minutes at or past this value count towards the duty cycle: how much of the window the label spent somewhere it should not stay. More than a rare minute past it also makes a label worth opening.</t>
+          <t>The fraction of retained minute summaries at or past this reference. It is a descriptive threshold crossing, not continuous elapsed duration, incident impact or proof of failure.</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The labels read beside this one, over the same seconds, when it is opened.</t>
+          <t>Other labels read over the selected observed sample window; navigation links, not causal claims.</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>What one second is</t>
+          <t>Sample formula</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
@@ -702,12 +702,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Share of the whole machine's CPU doing work: user, system, interrupts and steal, not idle and not waiting on I/O. Read on the minute's mean, which is how loaded the machine was; the seconds it spent pinned at the top are cpu.saturated. Past about 90% runnable threads queue for a core and every operation's latency grows with the queue.</t>
+          <t>Share of host CPU counters recorded as user, nice, system, IRQ, soft IRQ or steal, excluding idle and iowait; steal is not process execution time. Host-wide memory or CPU counters do not establish a container's resource limit. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, every second</t>
+          <t>Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>idle ≤5 (fading to 15) · low 15–35 (edges 5, 50) · moderate 50–65 (edges 35, 80) · high 80–88 (edges 65, 95) · saturated ≥95 (from 88)</t>
+          <t>idle ≤5 (fading to 15) · low 15–35 (edges 5, 50) · moderate 50–65 (edges 35, 80) · high 80–88 (edges 65, 95) · very_high ≥95 (from 88)</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>high or saturated</t>
+          <t>high or very_high</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Seconds the CPU was saturated</t>
+          <t>CPU-busy samples above 95%</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the whole machine's CPU was 95% busy or more. A minute mean of 50% can be thirty seconds pinned and thirty idle; this is the thirty. Operations that arrive in those seconds wait for a core.</t>
+          <t>Share of valid samples with the signal strictly above 95 %, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, every second</t>
+          <t>Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 95 %</t>
+          <t>valid-sample share strictly above 95 %, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>CPU waiting on I/O</t>
+          <t>Host CPU iowait share</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -846,12 +846,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Share of the machine's CPU idle with I/O outstanding. It says the processors had nothing to do but wait for storage; read it beside disk busy and disk await, which say which device.</t>
+          <t>Share of the machine's CPU idle with I/O outstanding. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/cpu/iowait_ms ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, every second</t>
+          <t>ΔsystemMetrics/cpu/iowait_ms ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CPU stolen by the hypervisor</t>
+          <t>Host CPU steal-time share</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -918,12 +918,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Share of the machine's CPU a virtual machine was ready to use and the hypervisor gave to someone else. Any sustained steal is a noisy neighbour or an oversubscribed host, and mongod cannot see it.</t>
+          <t>Share of the host CPU counters recorded as steal time. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/cpu/steal_ms ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, every second</t>
+          <t>ΔsystemMetrics/cpu/steal_ms ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/nice_ms + systemMetrics/cpu/system_ms + systemMetrics/cpu/idle_ms + systemMetrics/cpu/iowait_ms + systemMetrics/cpu/irq_ms + systemMetrics/cpu/softirq_ms + systemMetrics/cpu/steal_ms) × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>System CPU as a share of user plus system. mongod spends most of its CPU in user space; when the kernel takes as much or more, something below the database is working hard — TLS in the crypto library, transparent huge page compaction, reclaim under memory pressure, or a flood of small I/O. Read it beside cpu.busy: a high share of an idle machine means little.</t>
+          <t>System CPU as a share of user plus system. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/cpu/system_ms ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/system_ms) × 100, in %, every second; minutes where the divisor sums to under 6000 are left out</t>
+          <t>ΔsystemMetrics/cpu/system_ms ÷ Δ(systemMetrics/cpu/user_ms + systemMetrics/cpu/system_ms) × 100, in %, at each available sample; minutes where the divisor sums to under 6000 are left out</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Threads ready to run, per logical core, averaged over the minute. Above one, threads wait for a CPU and every operation queues behind them even when cpu.busy looks moderate on a many-core host.</t>
+          <t>Threads ready to run, per logical core, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>systemMetrics/cpu/procs_running ÷ systemMetrics/cpu/num_logical_cores, in per core, every second</t>
+          <t>systemMetrics/cpu/procs_running ÷ systemMetrics/cpu/num_logical_cores, in per core, at each available sample</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>light ≤0.5 (fading to 0.8) · busy 0.8–1.2 (edges 0.5, 2) · overloaded ≥2 (from 1.2)</t>
+          <t>light ≤0.5 (fading to 0.8) · busy 0.8–1.2 (edges 0.5, 2) · very_high ≥2 (from 1.2)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>overloaded</t>
+          <t>very_high</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Threads ready to run, per logical core, averaged over the minute. Above one, threads wait for a CPU and every operation queues behind them even when cpu.busy looks moderate on a many-core host.</t>
+          <t>Threads ready to run, per logical core, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>systemMetrics/cpu/procs_running ÷ systemMetrics/cpu/num_cpus, in per core, every second</t>
+          <t>systemMetrics/cpu/procs_running ÷ systemMetrics/cpu/num_cpus, in per core, at each available sample</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>light ≤0.5 (fading to 0.8) · busy 0.8–1.2 (edges 0.5, 2) · overloaded ≥2 (from 1.2)</t>
+          <t>light ≤0.5 (fading to 0.8) · busy 0.8–1.2 (edges 0.5, 2) · very_high ≥2 (from 1.2)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>overloaded</t>
+          <t>very_high</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Threads blocked on I/O</t>
+          <t>Processes in uninterruptible sleep</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Processes in uninterruptible sleep, averaged over the minute — almost always waiting on storage. A sustained handful means the disk is behind; it is also how a hung network mount shows, and FTDC itself can stop when its own statfs call blocks on one.</t>
+          <t>Host process count recorded in procs_blocked (uninterruptible sleep). Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>systemMetrics/cpu/procs_blocked, in threads, every second</t>
+          <t>systemMetrics/cpu/procs_blocked, in threads, at each available sample</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1278,12 +1278,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Context switches a second, host-wide. There is no level that is high for every machine; a step or a burst is threads contending — lock or spinlock contention, a connection storm.</t>
+          <t>Context switches a second, host-wide. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/cpu/ctxt per second, in /s, every second</t>
+          <t>ΔsystemMetrics/cpu/ctxt per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Share of the machine's memory not available to new allocations (MemTotal less MemAvailable, so the page cache the kernel can drop counts as free). Near the top the kernel reclaims hard, then the OOM killer chooses a process, and mongod is usually the largest. MongoDB collects MemAvailable from 4.2.14 and 4.4.5 (ftdc_system_stats_linux.cpp kMemKeys); earlier nodes do not get this label.</t>
+          <t>Share of the machine's memory not available to new allocations (MemTotal less MemAvailable, so the page cache the kernel can drop counts as free). Host-wide memory or CPU counters do not establish a container's resource limit. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>100 − (systemMetrics/memory/MemAvailable_kb ÷ systemMetrics/memory/MemTotal_kb × 100), in %, every second</t>
+          <t>100 − (systemMetrics/memory/MemAvailable_kb ÷ systemMetrics/memory/MemTotal_kb × 100), in %, at each available sample</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>low ≤40 (fading to 60) · moderate 60–75 (edges 40, 85) · high 85–92 (edges 75, 96) · exhausted ≥96 (from 92)</t>
+          <t>low ≤40 (fading to 60) · moderate 60–75 (edges 40, 85) · high 85–92 (edges 75, 96) · very_high ≥96 (from 92)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>high or exhausted</t>
+          <t>high or very_high</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Share of swap holding pages. A database whose pages are swapped out pays a disk read for memory it believes it has; any sustained swap on a mongod host is worth explaining, and swappiness or a cache sized past the container is the usual reason.</t>
+          <t>Share of swap holding pages. Host-wide memory or CPU counters do not establish a container's resource limit. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>100 − (systemMetrics/memory/SwapFree_kb ÷ systemMetrics/memory/SwapTotal_kb × 100), in %, every second</t>
+          <t>100 − (systemMetrics/memory/SwapFree_kb ÷ systemMetrics/memory/SwapTotal_kb × 100), in %, at each available sample</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1486,12 +1486,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Major page faults mongod took a second: memory it had to read back from disk. A burst is memory pressure — swap, or a page cache too small for what is read from it.</t>
+          <t>Rate of the process's logged major-page-fault counter. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/extra_info/page_faults per second, in /s, every second</t>
+          <t>ΔserverStatus/extra_info/page_faults per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>mongod's resident memory as a share of the machine's. In a container, compare it with the cgroup limit the log reports at startup, not with the host: a cache sized from host memory in a smaller container is a common cause of OOM kills.</t>
+          <t>mongod's resident memory as a share of the machine's. Host-wide memory or CPU counters do not establish a container's resource limit. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/mem/resident ÷ systemMetrics/memory/MemTotal_kb × 102400, in %, every second</t>
+          <t>serverStatus/mem/resident ÷ systemMetrics/memory/MemTotal_kb × 102400, in %, at each available sample</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Heap outside the WiredTiger cache</t>
+          <t>Allocated bytes minus WiredTiger cache bytes</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Bytes tcmalloc has allocated beyond what the WiredTiger cache holds: connections, sorts, aggregations, plan caches and fragmentation. Rising while the cache stays flat is the shape a reported memory leak usually has — and it is usually workload or allocator retention, not a leak.</t>
+          <t>Difference between tcmalloc allocated bytes and bytes currently held in the WiredTiger cache; this is a derived estimate, not a complete inventory of non-cache allocations. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/tcmalloc/generic/current_allocated_bytes − serverStatus/wiredTiger/cache/bytes currently in the cache × 9.313225746154785e-10, in GiB, every second</t>
+          <t>serverStatus/tcmalloc/generic/current_allocated_bytes − serverStatus/wiredTiger/cache/bytes currently in the cache × 9.313225746154785e-10, in GiB, at each available sample</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Memory freed but kept by tcmalloc</t>
+          <t>tcmalloc pageheap-free share</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Share of tcmalloc's heap that is free but not returned to the operating system (pageheap_free_bytes over heap_size). A large share is memory the machine counts against mongod that no operation is using; tcmallocReleaseRate decides how fast it goes back. Before 8.0 only: 8.0 Linux builds use Google tcmalloc, which keeps most free memory in per-CPU caches that pageheap_free_bytes does not count.</t>
+          <t>Ratio of tcmalloc pageheap_free_bytes to heap_size; these counters do not describe every allocator cache. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/tcmalloc/tcmalloc/pageheap_free_bytes ÷ serverStatus/tcmalloc/generic/heap_size × 100, in %, every second</t>
+          <t>serverStatus/tcmalloc/tcmalloc/pageheap_free_bytes ÷ serverStatus/tcmalloc/generic/heap_size × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1766,12 +1766,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>The configured cache as a share of the machine's memory. The default is half of RAM less a gigabyte; much more than that leaves too little for connections, sorts and the page cache. In a container the machine's memory may not be the limit the process lives under.</t>
+          <t>The configured cache as a share of the machine's memory. Host-wide memory or CPU counters do not establish a container's resource limit. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/cache/maximum bytes configured ÷ systemMetrics/memory/MemTotal_kb × 0.09765625, in %, every second</t>
+          <t>serverStatus/wiredTiger/cache/maximum bytes configured ÷ systemMetrics/memory/MemTotal_kb × 0.09765625, in %, at each available sample</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1786,17 +1786,17 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>conservative ≤30 (fading to 40) · default 40–55 (edges 30, 62) · oversized ≥70 (from 58)</t>
+          <t>low ≤30 (fading to 40) · middle 40–55 (edges 30, 62) · high ≥70 (from 58)</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>35 % → 50% conservative, 50% default</t>
+          <t>35 % → 50% low, 50% middle</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>oversized</t>
+          <t>high</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1838,12 +1838,12 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Share of each minute a block device had a request in flight (io_time). On a single spindle 100% is the limit; an SSD or a cloud volume serves many requests at once and can be 100% busy with room to spare, so read it beside disk await, which says whether requests actually waited. FTDC lists only devices with a /sys/block/&lt;dev&gt;/device entry, fixed at startup: dm-* (LVM) and md arrays are not there, only their member disks.</t>
+          <t>Device io_time counter advance divided by elapsed time; a high value does not establish device capacity exhaustion. Device coverage depends on the block-device counters present in FTDC; logical devices may be absent. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/disks/{i}/io_time_ms per second × 0.1, in %, every second; real block devices only</t>
+          <t>ΔsystemMetrics/disks/{i}/io_time_ms per second × 0.1, in %, at each available sample; real block devices only</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>idle ≤5 (fading to 15) · low 15–40 (edges 5, 60) · moderate 60–75 (edges 40, 85) · high 85–92 (edges 75, 97) · saturated ≥97 (from 92)</t>
+          <t>idle ≤5 (fading to 15) · low 15–40 (edges 5, 60) · moderate 60–75 (edges 40, 85) · high 85–92 (edges 75, 97) · very_high ≥97 (from 92)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>high or saturated</t>
+          <t>high or very_high</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Seconds the disk was saturated</t>
+          <t>Device-busy samples above 95%</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute a device was busy 95% of the second or more. A checkpoint that pins a volume for twenty seconds a minute averages to a third busy; this counts the twenty. Read it beside disk await: an SSD can be pinned and still answer fast.</t>
+          <t>Share of valid samples with the signal strictly above 95 %, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/disks/{i}/io_time_ms per second × 0.1, in %, every second; real block devices only</t>
+          <t>ΔsystemMetrics/disks/{i}/io_time_ms per second × 0.1, in %, at each available sample; real block devices only</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 95 %</t>
+          <t>valid-sample share strictly above 95 %, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1982,12 +1982,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Average milliseconds a read or write took on each device, queueing included — what iostat calls await. A local SSD answers in under a millisecond and a cloud volume in one to a few; tens of milliseconds means requests are waiting on the device or its throughput limit. Minutes with fewer than sixty requests are left out.</t>
+          <t>Average milliseconds a read or write took on each device, queueing included — what iostat calls await. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Δ(systemMetrics/disks/{i}/read_time_ms + systemMetrics/disks/{i}/write_time_ms) ÷ Δ(systemMetrics/disks/{i}/reads + systemMetrics/disks/{i}/writes), in ms, every second; minutes where the divisor sums to under 60 are left out; real block devices only</t>
+          <t>Δ(systemMetrics/disks/{i}/read_time_ms + systemMetrics/disks/{i}/write_time_ms) ÷ Δ(systemMetrics/disks/{i}/reads + systemMetrics/disks/{i}/writes), in ms, at each available sample; minutes where the divisor sums to under 60 are left out; real block devices only</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Average milliseconds a read took on each device. Slow reads with a quiet write side point at a cache too small for the working set; slow reads only during a snapshot or backup window point at whatever else was reading the volume.</t>
+          <t>Average milliseconds a read took on each device. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/disks/{i}/read_time_ms ÷ ΔsystemMetrics/disks/{i}/reads, in ms, every second; minutes where the divisor sums to under 60 are left out; real block devices only</t>
+          <t>ΔsystemMetrics/disks/{i}/read_time_ms ÷ ΔsystemMetrics/disks/{i}/reads, in ms, at each available sample; minutes where the divisor sums to under 60 are left out; real block devices only</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -2126,12 +2126,12 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Average milliseconds a write took on each device. Journal and checkpoint writes wait on it; slow writes are what turn a checkpoint into a stall and drain the write tickets.</t>
+          <t>Average milliseconds a write took on each device. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/disks/{i}/write_time_ms ÷ ΔsystemMetrics/disks/{i}/writes, in ms, every second; minutes where the divisor sums to under 60 are left out; real block devices only</t>
+          <t>ΔsystemMetrics/disks/{i}/write_time_ms ÷ ΔsystemMetrics/disks/{i}/writes, in ms, at each available sample; minutes where the divisor sums to under 60 are left out; real block devices only</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -2198,12 +2198,12 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Average number of requests outstanding on each device over the minute (io_queued time over wall time). A deep queue on a device that is also slow per request is a device at its limit; a deep queue answered fast is a device built for it.</t>
+          <t>Average number of requests outstanding on each device over the minute (io_queued time over wall time). Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/disks/{i}/io_queued_ms per second × 0.001, in requests, every second; real block devices only</t>
+          <t>ΔsystemMetrics/disks/{i}/io_queued_ms per second × 0.001, in requests, at each available sample; real block devices only</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Reads plus writes a second on each device. No level is high for every volume; a flat ceiling that busy and await press against is a provisioned IOPS limit or exhausted burst credits.</t>
+          <t>Reads plus writes a second on each device. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Δ(systemMetrics/disks/{i}/reads + systemMetrics/disks/{i}/writes) per second, in /s, every second; real block devices only</t>
+          <t>Δ(systemMetrics/disks/{i}/reads + systemMetrics/disks/{i}/writes) per second, in /s, at each available sample; real block devices only</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -2334,12 +2334,12 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Megabytes a second read plus written on each device (sectors are 512 bytes). A volume that is busy at low IOPS and high throughput is at its bandwidth limit rather than its request limit.</t>
+          <t>Megabytes a second read plus written on each device (sectors are 512 bytes). Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Δ(systemMetrics/disks/{i}/read_sectors + systemMetrics/disks/{i}/write_sectors) per second × 0.000512, in MB/s, every second; real block devices only</t>
+          <t>Δ(systemMetrics/disks/{i}/read_sectors + systemMetrics/disks/{i}/write_sectors) per second × 0.000512, in MB/s, at each available sample; real block devices only</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -2398,12 +2398,12 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Share of TCP segments the host sent again because the first copy was not acknowledged in time, across every connection on the machine. Above about one percent replication, heartbeats and client replies all slow down, and mongod has no counter of its own that shows it. Minutes that sent fewer than a thousand segments are left out.</t>
+          <t>Ratio of the host TCP RetransSegs counter advance to the OutSegs counter advance, across host connections. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/netstat/Tcp:RetransSegs ÷ ΔsystemMetrics/netstat/Tcp:OutSegs × 100, in %, every second; minutes where the divisor sums to under 1000 are left out</t>
+          <t>ΔsystemMetrics/netstat/Tcp:RetransSegs ÷ ΔsystemMetrics/netstat/Tcp:OutSegs × 100, in %, at each available sample; minutes where the divisor sums to under 1000 are left out</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -2418,17 +2418,17 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>clean ≤0.1 (fading to 0.3) · minor 0.3–0.7 (edges 0.1, 1) · lossy 1–2 (edges 0.7, 3) · severe ≥3 (from 2)</t>
+          <t>low ≤0.1 (fading to 0.3) · moderate 0.3–0.7 (edges 0.1, 1) · high 1–2 (edges 0.7, 3) · very_high ≥3 (from 2)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>0.2 % → 50% clean, 50% minor</t>
+          <t>0.2 % → 50% low, 50% moderate</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>lossy or severe</t>
+          <t>high or very_high</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Connections the kernel dropped a second because mongod's accept queue was full. A client refused here leaves nothing in the server log; any at all is worth explaining.</t>
+          <t>Rate of the host TCP ListenOverflows counter; the counter does not identify a MongoDB connection or client outcome. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/netstat/TcpExt:ListenOverflows per second, in /s, every second</t>
+          <t>ΔsystemMetrics/netstat/TcpExt:ListenOverflows per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -2542,12 +2542,12 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Established connections reset a second, host-wide. A burst is clients or a load balancer tearing connections down — timeouts, a failover, a proxy recycling its pool.</t>
+          <t>Established connections reset a second, host-wide. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>ΔsystemMetrics/netstat/Tcp:EstabResets per second, in /s, every second</t>
+          <t>ΔsystemMetrics/netstat/Tcp:EstabResets per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -2606,12 +2606,12 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Bytes a second in and out of mongod, from its own counters. Shape only: a step is a workload change, a periodic burst a job, and a ceiling the link or an instance's bandwidth limit.</t>
+          <t>Sum of the server's bytesIn and bytesOut counter rates, scaled to MB/s. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Δ(serverStatus/network/bytesIn + serverStatus/network/bytesOut) per second × 1e-06, in MB/s, every second</t>
+          <t>Δ(serverStatus/network/bytesIn + serverStatus/network/bytesOut) per second × 1e-06, in MB/s, at each available sample</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -2670,12 +2670,12 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Read tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. It is the general load on the pool: half used is worth noticing even when nothing ran out. Whether it ran out is tickets.read.scarce and tickets.read.empty; whether the pool itself changed size is tickets.read.pool.</t>
+          <t>Read tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/read/out ÷ serverStatus/wiredTiger/concurrentTransactions/read/totalTickets × 100, in %, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/read/out ÷ serverStatus/wiredTiger/concurrentTransactions/read/totalTickets × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Seconds with under 10% of read tickets left</t>
+          <t>Samples with under 10% of read tickets left</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -2742,17 +2742,17 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute fewer than a tenth of the read ticket pool was available, measured against the pool as it was that second, so it means the same thing for a pool the server resized as for a fixed one. Near-empty is where reads start to wait; a minute mean of the pool hides ten seconds of it entirely.</t>
+          <t>Share of valid samples with the signal strictly below 10 % available, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/read/available ÷ serverStatus/wiredTiger/concurrentTransactions/read/totalTickets × 100, in % available, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/read/available ÷ serverStatus/wiredTiger/concurrentTransactions/read/totalTickets × 100, in % available, at each available sample</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 10 % available</t>
+          <t>valid-sample share strictly below 10 % available, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Seconds with no read ticket left</t>
+          <t>Samples with no read ticket left</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2814,17 +2814,17 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the read ticket pool had none available. Every read that arrived in those seconds waited at the door of the storage engine. Reads waiting here are held behind whatever holds the tickets: long scans, slow reads from disk, eviction.</t>
+          <t>Share of valid samples with the signal strictly below 0.5 tickets left, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/read/available, in tickets left, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/read/available, in tickets left, at each available sample</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 0.5 tickets left</t>
+          <t>valid-sample share strictly below 0.5 tickets left, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2886,12 +2886,12 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>How many read tickets the pool held, averaged over the minute. Fixed unless someone changed it or, from 7.0, the server resized it to the load it measured; a step or an episode here is the pool growing under load or shrinking after it. Shape only: there is no size that is wrong for every server.</t>
+          <t>How many read tickets the pool held, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/read/totalTickets, in tickets, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/read/totalTickets, in tickets, at each available sample</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Milliseconds a second operations spent queued for a read ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. Not reported before 7.0. Reads waiting here are held behind whatever holds the tickets: long scans, slow reads from disk, eviction.</t>
+          <t>Milliseconds a second operations spent queued for a read ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/wiredTiger/concurrentTransactions/read/totalTimeQueuedMicros per second × 0.001, in ms/s, every second</t>
+          <t>ΔserverStatus/wiredTiger/concurrentTransactions/read/totalTimeQueuedMicros per second × 0.001, in ms/s, at each available sample</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -3022,12 +3022,12 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Read tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. It is the general load on the pool: half used is worth noticing even when nothing ran out. Whether it ran out is tickets.read.scarce and tickets.read.empty; whether the pool itself changed size is tickets.read.pool.</t>
+          <t>Read tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/read/out ÷ serverStatus/queues/execution/read/totalTickets × 100, in %, every second</t>
+          <t>serverStatus/queues/execution/read/out ÷ serverStatus/queues/execution/read/totalTickets × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Seconds with under 10% of read tickets left</t>
+          <t>Samples with under 10% of read tickets left</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -3094,17 +3094,17 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute fewer than a tenth of the read ticket pool was available, measured against the pool as it was that second, so it means the same thing for a pool the server resized as for a fixed one. Near-empty is where reads start to wait; a minute mean of the pool hides ten seconds of it entirely.</t>
+          <t>Share of valid samples with the signal strictly below 10 % available, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/read/available ÷ serverStatus/queues/execution/read/totalTickets × 100, in % available, every second</t>
+          <t>serverStatus/queues/execution/read/available ÷ serverStatus/queues/execution/read/totalTickets × 100, in % available, at each available sample</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 10 % available</t>
+          <t>valid-sample share strictly below 10 % available, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Seconds with no read ticket left</t>
+          <t>Samples with no read ticket left</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -3166,17 +3166,17 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the read ticket pool had none available. Every read that arrived in those seconds waited at the door of the storage engine. Reads waiting here are held behind whatever holds the tickets: long scans, slow reads from disk, eviction.</t>
+          <t>Share of valid samples with the signal strictly below 0.5 tickets left, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/read/available, in tickets left, every second</t>
+          <t>serverStatus/queues/execution/read/available, in tickets left, at each available sample</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 0.5 tickets left</t>
+          <t>valid-sample share strictly below 0.5 tickets left, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -3238,12 +3238,12 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>How many read tickets the pool held, averaged over the minute. Fixed unless someone changed it or, from 7.0, the server resized it to the load it measured; a step or an episode here is the pool growing under load or shrinking after it. Shape only: there is no size that is wrong for every server.</t>
+          <t>How many read tickets the pool held, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/read/totalTickets, in tickets, every second</t>
+          <t>serverStatus/queues/execution/read/totalTickets, in tickets, at each available sample</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -3302,12 +3302,12 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Milliseconds a second operations spent queued for a read ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. Not reported before 7.0. Reads waiting here are held behind whatever holds the tickets: long scans, slow reads from disk, eviction. Normal-priority operations only: exempt operations bypass the pool and are not counted.</t>
+          <t>Milliseconds a second operations spent queued for a read ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. The counter covers normal-priority operations, not exempt operations. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/queues/execution/read/normalPriority/totalTimeQueuedMicros per second × 0.001, in ms/s, every second</t>
+          <t>ΔserverStatus/queues/execution/read/normalPriority/totalTimeQueuedMicros per second × 0.001, in ms/s, at each available sample</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -3374,12 +3374,12 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Write tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. It is the general load on the pool: half used is worth noticing even when nothing ran out. Whether it ran out is tickets.write.scarce and tickets.write.empty; whether the pool itself changed size is tickets.write.pool.</t>
+          <t>Write tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/write/out ÷ serverStatus/wiredTiger/concurrentTransactions/write/totalTickets × 100, in %, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/write/out ÷ serverStatus/wiredTiger/concurrentTransactions/write/totalTickets × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Seconds with under 10% of write tickets left</t>
+          <t>Samples with under 10% of write tickets left</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -3446,17 +3446,17 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute fewer than a tenth of the write ticket pool was available, measured against the pool as it was that second, so it means the same thing for a pool the server resized as for a fixed one. Near-empty is where writes start to wait; a minute mean of the pool hides ten seconds of it entirely.</t>
+          <t>Share of valid samples with the signal strictly below 10 % available, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/write/available ÷ serverStatus/wiredTiger/concurrentTransactions/write/totalTickets × 100, in % available, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/write/available ÷ serverStatus/wiredTiger/concurrentTransactions/write/totalTickets × 100, in % available, at each available sample</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 10 % available</t>
+          <t>valid-sample share strictly below 10 % available, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Seconds with no write ticket left</t>
+          <t>Samples with no write ticket left</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -3518,17 +3518,17 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the write ticket pool had none available. Every write that arrived in those seconds waited at the door of the storage engine. Writes waiting here are usually behind checkpoints, dirty cache eviction or slow journal writes.</t>
+          <t>Share of valid samples with the signal strictly below 0.5 tickets left, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/write/available, in tickets left, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/write/available, in tickets left, at each available sample</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 0.5 tickets left</t>
+          <t>valid-sample share strictly below 0.5 tickets left, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>How many write tickets the pool held, averaged over the minute. Fixed unless someone changed it or, from 7.0, the server resized it to the load it measured; a step or an episode here is the pool growing under load or shrinking after it. Shape only: there is no size that is wrong for every server.</t>
+          <t>How many write tickets the pool held, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/concurrentTransactions/write/totalTickets, in tickets, every second</t>
+          <t>serverStatus/wiredTiger/concurrentTransactions/write/totalTickets, in tickets, at each available sample</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -3654,12 +3654,12 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Milliseconds a second operations spent queued for a write ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. Not reported before 7.0. Writes waiting here are usually behind checkpoints, dirty cache eviction or slow journal writes.</t>
+          <t>Milliseconds a second operations spent queued for a write ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/wiredTiger/concurrentTransactions/write/totalTimeQueuedMicros per second × 0.001, in ms/s, every second</t>
+          <t>ΔserverStatus/wiredTiger/concurrentTransactions/write/totalTimeQueuedMicros per second × 0.001, in ms/s, at each available sample</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -3726,12 +3726,12 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Write tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. It is the general load on the pool: half used is worth noticing even when nothing ran out. Whether it ran out is tickets.write.scarce and tickets.write.empty; whether the pool itself changed size is tickets.write.pool.</t>
+          <t>Write tickets in use as a share of the pool as it was that second (out over totalTickets), averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/write/out ÷ serverStatus/queues/execution/write/totalTickets × 100, in %, every second</t>
+          <t>serverStatus/queues/execution/write/out ÷ serverStatus/queues/execution/write/totalTickets × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Seconds with under 10% of write tickets left</t>
+          <t>Samples with under 10% of write tickets left</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -3798,17 +3798,17 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute fewer than a tenth of the write ticket pool was available, measured against the pool as it was that second, so it means the same thing for a pool the server resized as for a fixed one. Near-empty is where writes start to wait; a minute mean of the pool hides ten seconds of it entirely.</t>
+          <t>Share of valid samples with the signal strictly below 10 % available, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/write/available ÷ serverStatus/queues/execution/write/totalTickets × 100, in % available, every second</t>
+          <t>serverStatus/queues/execution/write/available ÷ serverStatus/queues/execution/write/totalTickets × 100, in % available, at each available sample</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 10 % available</t>
+          <t>valid-sample share strictly below 10 % available, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Seconds with no write ticket left</t>
+          <t>Samples with no write ticket left</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the write ticket pool had none available. Every write that arrived in those seconds waited at the door of the storage engine. Writes waiting here are usually behind checkpoints, dirty cache eviction or slow journal writes.</t>
+          <t>Share of valid samples with the signal strictly below 0.5 tickets left, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/write/available, in tickets left, every second</t>
+          <t>serverStatus/queues/execution/write/available, in tickets left, at each available sample</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 0.5 tickets left</t>
+          <t>valid-sample share strictly below 0.5 tickets left, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -3942,12 +3942,12 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>How many write tickets the pool held, averaged over the minute. Fixed unless someone changed it or, from 7.0, the server resized it to the load it measured; a step or an episode here is the pool growing under load or shrinking after it. Shape only: there is no size that is wrong for every server.</t>
+          <t>How many write tickets the pool held, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/queues/execution/write/totalTickets, in tickets, every second</t>
+          <t>serverStatus/queues/execution/write/totalTickets, in tickets, at each available sample</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -4006,12 +4006,12 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Milliseconds a second operations spent queued for a write ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. Not reported before 7.0. Writes waiting here are usually behind checkpoints, dirty cache eviction or slow journal writes. Normal-priority operations only: exempt operations bypass the pool and are not counted.</t>
+          <t>Milliseconds a second operations spent queued for a write ticket, added across every operation waiting: 1000 is one operation waiting the whole second, or ten waiting a tenth of it. The counter covers normal-priority operations, not exempt operations. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/queues/execution/write/normalPriority/totalTimeQueuedMicros per second × 0.001, in ms/s, every second</t>
+          <t>ΔserverStatus/queues/execution/write/normalPriority/totalTimeQueuedMicros per second × 0.001, in ms/s, at each available sample</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Seconds with reads queued</t>
+          <t>Samples with reads queued</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -4078,17 +4078,17 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute at least one read operation was queued for a lock or a ticket (globalLock.currentQueue.readers). How deep the queue got is the label's peak second.</t>
+          <t>Share of valid samples with the signal strictly above 0 operations, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/globalLock/currentQueue/readers, in operations, every second</t>
+          <t>serverStatus/globalLock/currentQueue/readers, in operations, at each available sample</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 0 operations</t>
+          <t>valid-sample share strictly above 0 operations, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Seconds with writes queued</t>
+          <t>Samples with writes queued</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -4150,17 +4150,17 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute at least one write operation was queued for a lock or a ticket (globalLock.currentQueue.writers). How deep the queue got is the label's peak second.</t>
+          <t>Share of valid samples with the signal strictly above 0 operations, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/globalLock/currentQueue/writers, in operations, every second</t>
+          <t>serverStatus/globalLock/currentQueue/writers, in operations, at each available sample</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 0 operations</t>
+          <t>valid-sample share strictly above 0 operations, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -4222,12 +4222,12 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Bytes in the WiredTiger cache as a share of its configured size, averaged over the minute. Eviction keeps it near 80%; at 95% (eviction_trigger) application threads are made to evict before they may proceed, which turns cache pressure into operation latency. The seconds spent past that line are cache.over_trigger.</t>
+          <t>Bytes in the WiredTiger cache as a share of its configured size, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/cache/bytes currently in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, every second</t>
+          <t>serverStatus/wiredTiger/cache/bytes currently in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>low ≤50 (fading to 70) · normal 70–80 (edges 50, 86) · high 86–93 (edges 80, 95) · over_trigger ≥96 (from 94)</t>
+          <t>low ≤50 (fading to 70) · normal 70–80 (edges 50, 86) · high 86–93 (edges 80, 95) · above_reference ≥96 (from 94)</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="K52" s="4" t="inlineStr">
         <is>
-          <t>high or over_trigger</t>
+          <t>high or above_reference</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Seconds the cache was past its eviction trigger</t>
+          <t>Cache-fill samples above 95%</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -4294,17 +4294,17 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the cache was 95% full or more — past eviction_trigger, where operations are made to evict pages themselves before they may go on. Each of those seconds is latency added to whatever ran in it.</t>
+          <t>Share of valid samples with the signal strictly above 95 %, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/cache/bytes currently in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, every second</t>
+          <t>serverStatus/wiredTiger/cache/bytes currently in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 95 %</t>
+          <t>valid-sample share strictly above 95 %, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -4366,12 +4366,12 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Modified bytes not yet written, as a share of the configured cache, averaged over the minute. Eviction aims for 5%; at 20% (eviction_dirty_trigger) application threads are made to write dirty pages out themselves, and the seconds spent there are cache.dirty_over_trigger. Sustained high dirty cache is a write load the disk or the checkpoint is not keeping up with. From 7.0 the targets can be set in gigabytes at startup (wiredTigerEvictionDirtyTargetGB, wiredTigerEvictionDirtyMaxGB), which moves these lines.</t>
+          <t>Modified bytes not yet written, as a share of the configured cache, averaged over the minute. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/cache/tracked dirty bytes in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, every second</t>
+          <t>serverStatus/wiredTiger/cache/tracked dirty bytes in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>low ≤3 (fading to 6) · normal 6–8 (edges 3, 12) · high 12–18 (edges 8, 20) · over_trigger ≥21 (from 19)</t>
+          <t>low ≤3 (fading to 6) · normal 6–8 (edges 3, 12) · high 12–18 (edges 8, 20) · above_reference ≥21 (from 19)</t>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr">
@@ -4396,7 +4396,7 @@
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>high or over_trigger</t>
+          <t>high or above_reference</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Seconds the dirty cache was past its trigger</t>
+          <t>Dirty-cache samples above 20%</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -4438,17 +4438,17 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute dirty data was 20% of the cache or more — past eviction_dirty_trigger, where operations are made to write dirty pages out themselves. Writes slow down in exactly these seconds, and the write tickets drain behind them.</t>
+          <t>Share of valid samples with the signal strictly above 20 %, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/cache/tracked dirty bytes in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, every second</t>
+          <t>serverStatus/wiredTiger/cache/tracked dirty bytes in the cache ÷ serverStatus/wiredTiger/cache/maximum bytes configured × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 20 %</t>
+          <t>valid-sample share strictly above 20 %, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -4510,12 +4510,12 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Pages a second that operations evicted themselves because the eviction workers could not keep the cache under its triggers. Each one is time a query or a write spent doing the storage engine's housekeeping instead of its own work.</t>
+          <t>Rate of pages evicted by application threads; where the version uses attempts and failures, the signal subtracts failure counts from attempt counts. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/wiredTiger/cache/pages evicted by application threads per second, in pages/s, every second</t>
+          <t>ΔserverStatus/wiredTiger/cache/pages evicted by application threads per second, in pages/s, at each available sample</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -4582,12 +4582,12 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Pages a second that operations evicted themselves because the eviction workers could not keep the cache under its triggers — read from 8.0.16 as the attempts that did not fail. Each one is time a query or a write spent doing the storage engine's housekeeping instead of its own work.</t>
+          <t>Rate of pages evicted by application threads; where the version uses attempts and failures, the signal subtracts failure counts from attempt counts. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/wiredTiger/cache/page evict attempts by application threads − serverStatus/wiredTiger/cache/page evict failures by application threads per second, in pages/s, every second</t>
+          <t>ΔserverStatus/wiredTiger/cache/page evict attempts by application threads − serverStatus/wiredTiger/cache/page evict failures by application threads per second, in pages/s, at each available sample</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -4654,12 +4654,12 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Milliseconds a second application threads spent evicting pages, added across every thread doing it (8.0 and later): 1000 is one operation spending the whole second on the storage engine's housekeeping. It is the latency cost of cache pressure, measured directly.</t>
+          <t>Application-thread eviction time counter advance per elapsed second, summed across threads, in milliseconds. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/wiredTiger/cache/application thread time evicting (usecs) per second × 0.001, in ms/s, every second</t>
+          <t>ΔserverStatus/wiredTiger/cache/application thread time evicting (usecs) per second × 0.001, in ms/s, at each available sample</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -4726,12 +4726,12 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Megabytes a second WiredTiger read from disk into its cache. A step up with the same workload is a working set that stopped fitting, or a new scan reading what was never hot.</t>
+          <t>WiredTiger bytes-read-into-cache counter advance per elapsed second, scaled to MB/s. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/wiredTiger/cache/bytes read into cache per second × 1e-06, in MB/s, every second</t>
+          <t>ΔserverStatus/wiredTiger/cache/bytes read into cache per second × 1e-06, in MB/s, at each available sample</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -4790,17 +4790,17 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Seconds the most recent WiredTiger checkpoint took, read on the longest the minute reported. Checkpoints start every 60 seconds; one that takes longer runs back to back with the next, and dirty data accumulates behind it.</t>
+          <t>Duration recorded for the most recent WiredTiger checkpoint; the same completed-checkpoint value may appear in multiple samples. Minute summaries select the highest valid sample. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/transaction/transaction checkpoint most recent time (msecs) × 0.001, in s, every second</t>
+          <t>serverStatus/wiredTiger/transaction/transaction checkpoint most recent time (msecs) × 0.001, in s, at each available sample</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>the highest second of each minute</t>
+          <t>the highest valid sample of each minute</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
@@ -4862,17 +4862,17 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Seconds the most recent WiredTiger checkpoint took, read on the longest the minute reported. Checkpoints start every 60 seconds; one that takes longer runs back to back with the next, and dirty data accumulates behind it.</t>
+          <t>Duration recorded for the most recent WiredTiger checkpoint; the same completed-checkpoint value may appear in multiple samples. Minute summaries select the highest valid sample. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/checkpoint/most recent time (msecs) × 0.001, in s, every second</t>
+          <t>serverStatus/wiredTiger/checkpoint/most recent time (msecs) × 0.001, in s, at each available sample</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>the highest second of each minute</t>
+          <t>the highest valid sample of each minute</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Seconds spent checkpointing</t>
+          <t>Samples with checkpoint activity</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -4934,17 +4934,17 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute a checkpoint was running. Checkpoints start every 60 seconds; near a full minute they run back to back, and dirty data piles up behind them.</t>
+          <t>Share of valid samples with the signal strictly above 0 running, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/transaction/transaction checkpoint currently running, in running, every second</t>
+          <t>serverStatus/wiredTiger/transaction/transaction checkpoint currently running, in running, at each available sample</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 0 running</t>
+          <t>valid-sample share strictly above 0 running, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Seconds spent checkpointing</t>
+          <t>Samples with checkpoint activity</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -5006,17 +5006,17 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute a checkpoint was running. Checkpoints start every 60 seconds; near a full minute they run back to back, and dirty data piles up behind them. From 7.1 WiredTiger reports a checkpoint progress state code instead (0 is inactive), read here as running whenever it is not zero.</t>
+          <t>Share of valid samples with the signal strictly above 0 state, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/checkpoint/progress state, in state, every second</t>
+          <t>serverStatus/wiredTiger/checkpoint/progress state, in state, at each available sample</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 0 state</t>
+          <t>valid-sample share strictly above 0 state, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -5078,12 +5078,12 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>WiredTiger data handles currently open: roughly one per collection and index in use. Climbing toward the open-file limit ends in "Too many open files" and a fatal WiredTiger panic; many collections and a periodic stats sweep across them is the usual way there.</t>
+          <t>Count reported by WiredTiger for currently open data handles. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/wiredTiger/data-handle/connection data handles currently active, in handles, every second</t>
+          <t>serverStatus/wiredTiger/data-handle/connection data handles currently active, in handles, at each available sample</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -5138,12 +5138,12 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Average milliseconds per read operation over each minute, from opLatencies: every microsecond spent on reads in the minute over every read that finished in it. Tailable getMores — a secondary or a change stream waiting for new oplog entries — count as reads and can hold this up on a healthy primary, so read it beside the slow query log. Minutes with fewer than sixty reads are left out.</t>
+          <t>Average milliseconds per read operation over each minute, from opLatencies: every microsecond spent on reads in the minute over every read that finished in it. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/opLatencies/reads/latency ÷ ΔserverStatus/opLatencies/reads/ops × 0.001, in ms, every second; minutes where the divisor sums to under 60 are left out</t>
+          <t>ΔserverStatus/opLatencies/reads/latency ÷ ΔserverStatus/opLatencies/reads/ops × 0.001, in ms, at each available sample; minutes where the divisor sums to under 60 are left out</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -5210,12 +5210,12 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Average milliseconds per write operation over each minute, from opLatencies. Minutes with fewer than sixty writes are left out.</t>
+          <t>Average milliseconds per write operation over each minute, from opLatencies. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/opLatencies/writes/latency ÷ ΔserverStatus/opLatencies/writes/ops × 0.001, in ms, every second; minutes where the divisor sums to under 60 are left out</t>
+          <t>ΔserverStatus/opLatencies/writes/latency ÷ ΔserverStatus/opLatencies/writes/ops × 0.001, in ms, at each available sample; minutes where the divisor sums to under 60 are left out</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -5282,12 +5282,12 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Average milliseconds per command over each minute, from opLatencies: everything that is not a CRUD read or write, aggregate included on most versions. Minutes with fewer than sixty commands are left out.</t>
+          <t>Ratio of command opLatencies counter advance to command operation-count advance, scaled to milliseconds per operation. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/opLatencies/commands/latency ÷ ΔserverStatus/opLatencies/commands/ops × 0.001, in ms, every second; minutes where the divisor sums to under 60 are left out</t>
+          <t>ΔserverStatus/opLatencies/commands/latency ÷ ΔserverStatus/opLatencies/commands/ops × 0.001, in ms, at each available sample; minutes where the divisor sums to under 60 are left out</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -5354,12 +5354,12 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>Every operation the server ran a second: queries, getMores, inserts, updates, deletes and commands. Shape only: a step is a new workload, a periodic burst a job or a batch.</t>
+          <t>Sum of query, getMore, insert, update, delete and command operation-counter rates. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Δ(serverStatus/opcounters/query + serverStatus/opcounters/getmore + serverStatus/opcounters/insert + serverStatus/opcounters/update + serverStatus/opcounters/delete + serverStatus/opcounters/command) per second, in ops/s, every second</t>
+          <t>Δ(serverStatus/opcounters/query + serverStatus/opcounters/getmore + serverStatus/opcounters/insert + serverStatus/opcounters/update + serverStatus/opcounters/delete + serverStatus/opcounters/command) per second, in ops/s, at each available sample</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -5418,12 +5418,12 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>Inserts, updates and deletes a second. A burst of writes is what fills the dirty cache and stretches checkpoints a few minutes later.</t>
+          <t>Sum of insert, update and delete operation-counter rates. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Δ(serverStatus/opcounters/insert + serverStatus/opcounters/update + serverStatus/opcounters/delete) per second, in ops/s, every second</t>
+          <t>Δ(serverStatus/opcounters/insert + serverStatus/opcounters/update + serverStatus/opcounters/delete) per second, in ops/s, at each available sample</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -5482,12 +5482,12 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Documents scanned for every document returned, across the server, over each minute. Near 1 queries are well indexed; in the hundreds or thousands something is scanning — a COLLSCAN or an index that does not cover the filter. The slow query log names which shape. Minutes that returned fewer than sixty documents are left out.</t>
+          <t>Ratio of documents-examined counter advance to documents-returned counter advance; it does not determine index suitability. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/metrics/queryExecutor/scannedObjects ÷ ΔserverStatus/metrics/document/returned, in ratio, every second; minutes where the divisor sums to under 60 are left out</t>
+          <t>ΔserverStatus/metrics/queryExecutor/scannedObjects ÷ ΔserverStatus/metrics/document/returned, in ratio, at each available sample; minutes where the divisor sums to under 60 are left out</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -5502,17 +5502,17 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>efficient ≤2 (fading to 10) · loose 10–50 (edges 2, 100) · scanning 100–500 (edges 50, 1000) · very_poor ≥1000 (from 500)</t>
+          <t>low ≤2 (fading to 10) · moderate 10–50 (edges 2, 100) · high 100–500 (edges 50, 1000) · very_high ≥1000 (from 500)</t>
         </is>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>6 ratio → 50% efficient, 50% loose</t>
+          <t>6 ratio → 50% low, 50% moderate</t>
         </is>
       </c>
       <c r="K70" s="4" t="inlineStr">
         <is>
-          <t>scanning or very_poor</t>
+          <t>high or very_high</t>
         </is>
       </c>
       <c r="L70" s="4" t="inlineStr">
@@ -5554,12 +5554,12 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Queries a second that read a whole collection (4.4 and later). Any steady rate on a large collection is a missing index; a burst is a report or a job.</t>
+          <t>Rate of the server's collection-scan counter. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/metrics/queryExecutor/collectionScans/total per second, in /s, every second</t>
+          <t>ΔserverStatus/metrics/queryExecutor/collectionScans/total per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>In-memory sorts</t>
+          <t>scanAndOrder counter rate</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -5626,12 +5626,12 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Operations a second that sorted in memory because no index gave the order (scanAndOrder). They cost CPU and memory and fail past the sort limit.</t>
+          <t>Rate of the server's scanAndOrder counter. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/metrics/operation/scanAndOrder per second, in /s, every second</t>
+          <t>ΔserverStatus/metrics/operation/scanAndOrder per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -5690,12 +5690,12 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Write conflicts a second: two operations updating the same document at once, one retrying. A burst means hot documents — a counter, a queue collection, a status field everyone updates.</t>
+          <t>Rate of the server's writeConflicts counter; retries, document identity and contention cause are not inferred from this counter. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/metrics/operation/writeConflicts per second, in /s, every second</t>
+          <t>ΔserverStatus/metrics/operation/writeConflicts per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -5762,12 +5762,12 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Documents the TTL monitor deleted a second. TTL runs every minute; a large expiry deletes in bursts that load the disk and the oplog, and nightly expiry is a classic periodic cause.</t>
+          <t>Rate of documents reported deleted by the TTL monitor; collection identity, expiry backlog and latency impact are not inferred. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/metrics/ttl/deletedDocuments per second, in docs/s, every second</t>
+          <t>ΔserverStatus/metrics/ttl/deletedDocuments per second, in docs/s, at each available sample</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -5826,12 +5826,12 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Cursors open on the server. A climb that never comes down is clients not closing or not exhausting cursors, and each one holds resources until it times out.</t>
+          <t>Count reported for currently open cursors. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/metrics/cursor/open/total, in cursors, every second</t>
+          <t>serverStatus/metrics/cursor/open/total, in cursors, at each available sample</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -5890,17 +5890,17 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>How many seconds each member's last applied write trailed the newest write any member had, as this node's replSetGetStatus reported them — one result per member, read on the worst second of each minute. A lagging member is usually short of disk or CPU, applying a large batch, or syncing across a slow link. Members are numbered by their place in the replica set config; an arbiter has no optime and gets no result. Before 6.0 optimeDate has one-second resolution.</t>
+          <t>Difference between each member's reported applied-write timestamp and the newest such timestamp in this node's replica-set status, scaled to seconds. Members without a timestamp have no result. optimeDate has one-second resolution. Minute summaries select the highest valid sample. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>newest of every replSetGetStatus/members/{i}/optimeDate − this one × 0.001, in s, every second</t>
+          <t>newest of every replSetGetStatus/members/{i}/optimeDate − this one × 0.001, in s, at each available sample</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>the highest second of each minute</t>
+          <t>the highest valid sample of each minute</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -5962,17 +5962,17 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>How many seconds each member's last applied write trailed the newest write any member had, as this node's replSetGetStatus reported them — one result per member, read on the worst second of each minute. A lagging member is usually short of disk or CPU, applying a large batch, or syncing across a slow link. Members are numbered by their place in the replica set config; an arbiter has no optime and gets no result.</t>
+          <t>Difference between each member's reported applied-write timestamp and the newest such timestamp in this node's replica-set status, scaled to seconds. Members without a timestamp have no result. Minute summaries select the highest valid sample. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>newest of every replSetGetStatus/members/{i}/lastAppliedWallTime − this one × 0.001, in s, every second</t>
+          <t>newest of every replSetGetStatus/members/{i}/lastAppliedWallTime − this one × 0.001, in s, at each available sample</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>the highest second of each minute</t>
+          <t>the highest valid sample of each minute</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -6034,17 +6034,17 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>Seconds between the newest write this node applied and the newest write a majority had (lastAppliedWallTime less lastCommittedWallTime), read on the worst second of each minute. It is what w:majority writes wait for and what flow control throttles on; it grows when enough secondaries fall behind.</t>
+          <t>Difference between this node's lastAppliedWallTime and lastCommittedWallTime, scaled to seconds. Minute summaries select the highest valid sample. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>replSetGetStatus/optimes/lastAppliedWallTime − replSetGetStatus/optimes/lastCommittedWallTime × 0.001, in s, every second</t>
+          <t>replSetGetStatus/optimes/lastAppliedWallTime − replSetGetStatus/optimes/lastCommittedWallTime × 0.001, in s, at each available sample</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>the highest second of each minute</t>
+          <t>the highest valid sample of each minute</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Seconds flow control was engaged</t>
+          <t>Samples with flowControl.isLagged set</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -6106,17 +6106,17 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute flow control reported the set lagged and limited writes on the primary. Any of it means writers were held back on purpose because the majority fell behind. Meaningful on a primary with flow control enabled; a secondary reports it unset.</t>
+          <t>Share of valid samples with the signal strictly above 0 lagged, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/flowControl/isLagged, in lagged, every second</t>
+          <t>serverStatus/flowControl/isLagged, in lagged, at each available sample</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 0 lagged</t>
+          <t>valid-sample share strictly above 0 lagged, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
@@ -6178,12 +6178,12 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>Milliseconds a second writes spent waiting for flow control tickets on this node, added across every write waiting.</t>
+          <t>Milliseconds a second writes spent waiting for flow control tickets on this node, added across every write waiting. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/flowControl/timeAcquiringMicros per second × 0.001, in ms/s, every second</t>
+          <t>ΔserverStatus/flowControl/timeAcquiringMicros per second × 0.001, in ms/s, at each available sample</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Operations a second this node applied from the oplog, as a secondary. A drop to nothing while the buffer holds entries is an applier that is stuck, not slow.</t>
+          <t>Rate of the node's oplog application operation counter. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/metrics/repl/apply/ops per second, in ops/s, every second</t>
+          <t>ΔserverStatus/metrics/repl/apply/ops per second, in ops/s, at each available sample</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
@@ -6314,12 +6314,12 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Share of the replication apply buffer in use on a secondary, averaged over the minute. Full, the node fetches faster than it applies — it is behind on disk or CPU, not on the network.</t>
+          <t>Reported replication buffer bytes as a share of its reported maximum. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/metrics/repl/buffer/sizeBytes ÷ serverStatus/metrics/repl/buffer/maxSizeBytes × 100, in %, every second</t>
+          <t>serverStatus/metrics/repl/buffer/sizeBytes ÷ serverStatus/metrics/repl/buffer/maxSizeBytes × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
@@ -6386,12 +6386,12 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Share of the replication apply buffer in use on a secondary, averaged over the minute. Full, the node fetches faster than it applies — it is behind on disk or CPU, not on the network.</t>
+          <t>Reported replication buffer bytes as a share of its reported maximum. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/metrics/repl/buffer/apply/sizeBytes ÷ serverStatus/metrics/repl/buffer/apply/maxSizeBytes × 100, in %, every second</t>
+          <t>serverStatus/metrics/repl/buffer/apply/sizeBytes ÷ serverStatus/metrics/repl/buffer/apply/maxSizeBytes × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Seconds the apply buffer was nearly full</t>
+          <t>Apply-buffer samples above 90%</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -6458,17 +6458,17 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the replication apply buffer was 90% full or more. While it is, the node stops fetching until the applier catches up.</t>
+          <t>Share of valid samples with the signal strictly above 90 %, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/metrics/repl/buffer/sizeBytes ÷ serverStatus/metrics/repl/buffer/maxSizeBytes × 100, in %, every second</t>
+          <t>serverStatus/metrics/repl/buffer/sizeBytes ÷ serverStatus/metrics/repl/buffer/maxSizeBytes × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 90 %</t>
+          <t>valid-sample share strictly above 90 %, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Seconds the apply buffer was nearly full</t>
+          <t>Apply-buffer samples above 90%</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -6530,17 +6530,17 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute the replication apply buffer was 90% full or more. While it is, the node stops fetching until the applier catches up.</t>
+          <t>Share of valid samples with the signal strictly above 90 %, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/metrics/repl/buffer/apply/sizeBytes ÷ serverStatus/metrics/repl/buffer/apply/maxSizeBytes × 100, in %, every second</t>
+          <t>serverStatus/metrics/repl/buffer/apply/sizeBytes ÷ serverStatus/metrics/repl/buffer/apply/maxSizeBytes × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute above 90 %</t>
+          <t>valid-sample share strictly above 90 %, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Connection limit in use</t>
+          <t>Current connections as a share of current plus available</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -6602,12 +6602,12 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Open connections as a share of the most the server will accept (current over current plus available), averaged over the minute. Near the limit new clients are refused, and the log says so; the seconds spent there are connections.scarce.</t>
+          <t>Reported current connections divided by current plus available connections. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/connections/current ÷ (serverStatus/connections/current + serverStatus/connections/available) × 100, in %, every second</t>
+          <t>serverStatus/connections/current ÷ (serverStatus/connections/current + serverStatus/connections/available) × 100, in %, at each available sample</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Seconds with under 10% of connections left</t>
+          <t>Samples with under 10% of connections left</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -6674,17 +6674,17 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Seconds of each minute fewer than a tenth of the connection limit was still available. A reconnect storm can hit the limit for a few seconds and leave a minute mean looking calm.</t>
+          <t>Share of valid samples with the signal strictly below 10 % available, normalized to a 60-second minute. This is a normalized sample share, not measured continuous elapsed duration; cadence and gaps must be checked. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/connections/available ÷ (serverStatus/connections/current + serverStatus/connections/available) × 100, in % available, every second</t>
+          <t>serverStatus/connections/available ÷ (serverStatus/connections/current + serverStatus/connections/available) × 100, in % available, at each available sample</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>seconds of each minute below 10 % available</t>
+          <t>valid-sample share strictly below 10 % available, normalized to 60 s/min; not continuous elapsed time</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -6746,12 +6746,12 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Connections opened a second. Drivers keep a pool, so a steady few is normal; tens a second is clients reconnecting, usually after timeouts, or an application opening a client per request. Each one costs the server a thread and an authentication.</t>
+          <t>Rate of the server's totalCreated connection counter. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/connections/totalCreated per second, in conn/s, every second</t>
+          <t>ΔserverStatus/connections/totalCreated per second, in conn/s, at each available sample</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>quiet ≤1 (fading to 3) · normal 3–10 (edges 1, 20) · storm ≥20 (from 10)</t>
+          <t>quiet ≤1 (fading to 3) · normal 3–10 (edges 1, 20) · high ≥20 (from 10)</t>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>storm</t>
+          <t>high</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Open connections doing nothing</t>
+          <t>Derived non-active connection count</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -6818,12 +6818,12 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Open connections with no operation in progress, leaving out drivers' monitoring connections, averaged over the minute. Most of a client pool is idle on any healthy server, so the share says little; the count is what costs: every connection holds a thread and memory on the server. Thousands of them is a pool sized far past what the workload uses, or one that grew during a stall and never shrank.</t>
+          <t>Derived connection count: current plus awaitingTopologyChanges minus active; it is not evidence of unused client pools or a connection leak. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>(serverStatus/connections/current + serverStatus/connections/awaitingTopologyChanges) − serverStatus/connections/active, in conns, every second</t>
+          <t>(serverStatus/connections/current + serverStatus/connections/awaitingTopologyChanges) − serverStatus/connections/active, in conns, at each available sample</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
@@ -6838,7 +6838,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>few ≤300 (fading to 800) · many 800–1500 (edges 300, 2500) · excessive ≥3000 (from 1500)</t>
+          <t>few ≤300 (fading to 800) · many 800–1500 (edges 300, 2500) · very_high ≥3000 (from 1500)</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="K89" s="4" t="inlineStr">
         <is>
-          <t>excessive</t>
+          <t>very_high</t>
         </is>
       </c>
       <c r="L89" s="4" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Open connections with an operation in progress</t>
+          <t>Derived active-connection share</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -6890,17 +6890,17 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>Share of the open connections with an operation in progress, leaving out drivers' monitoring connections, at the worst second of each minute. It stays low on a healthy server, because operations finish faster than they arrive; when the server stalls, every operation in flight waits and the share jumps. A pile-up here beside empty ticket pools or queued operations is a stall seen from the client side.</t>
+          <t>Derived active-connection share: active minus awaitingTopologyChanges divided by current connections. Minute summaries select the highest valid sample. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/connections/active − serverStatus/connections/awaitingTopologyChanges ÷ serverStatus/connections/current × 100, in %, every second; minutes where the divisor sums to under 3000 are left out</t>
+          <t>serverStatus/connections/active − serverStatus/connections/awaitingTopologyChanges ÷ serverStatus/connections/current × 100, in %, at each available sample; minutes where the divisor sums to under 3000 are left out</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>the highest second of each minute</t>
+          <t>the highest valid sample of each minute</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -6910,7 +6910,7 @@
       </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>calm ≤10 (fading to 25) · busy 25–40 (edges 10, 60) · piled_up ≥60 (from 40)</t>
+          <t>calm ≤10 (fading to 25) · busy 25–40 (edges 10, 60) · high ≥60 (from 40)</t>
         </is>
       </c>
       <c r="J90" s="4" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="K90" s="4" t="inlineStr">
         <is>
-          <t>piled_up</t>
+          <t>high</t>
         </is>
       </c>
       <c r="L90" s="4" t="inlineStr">
@@ -6962,12 +6962,12 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>Connections open to this node. Shape only — the limit is in connections.used. A step is a deployment or a pool resize; a climb that never comes down is a client leaking connections.</t>
+          <t>Count reported for currently open server connections. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>serverStatus/connections/current, in conns, every second</t>
+          <t>serverStatus/connections/current, in conns, at each available sample</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
@@ -7026,12 +7026,12 @@
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>Connections mongod refused a second because it was at its limit (6.3 and later). Each one is a client error the application saw.</t>
+          <t>Rate of the server's rejected connection counter; client impact and rejection cause are not inferred. Minute summaries use a ratio of sums for ratio signals and a mean otherwise. Numeric bands and thresholds are fixed descriptive references, not a diagnosis or a discovered server limit. Paired labels are navigation links, not causal claims.</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>ΔserverStatus/connections/rejected per second, in /s, every second</t>
+          <t>ΔserverStatus/connections/rejected per second, in /s, at each available sample</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">

</xml_diff>